<commit_message>
feat: tambahkan sheet 5. Timeline Humas dan simpan berkas notula rapat serta TOR LDKM 2026
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Pemateri Fix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Template Chat" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Koordinasi Kosma" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Timeline Humas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <color rgb="FF262626"/>
@@ -64,8 +65,20 @@
       <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +114,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -222,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -266,6 +291,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2238,12 +2269,12 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Belum Ada Jadwal</t>
+          <t>Selesai (Done)</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Rina</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2311,12 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Ada Jadwal</t>
+          <t>Selesai (Done)</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dina, Klar</t>
         </is>
       </c>
     </row>
@@ -2496,6 +2527,723 @@
       <c r="H12" s="17" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Pilar Kerja</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Program Kerja / Tugas Spesifik</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Rentang Waktu</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>PIC / Petugas</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Keterangan / Output yang Diharapkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Sosialisasi Maba</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>Pendataan Kontak Kosma 11 Jurusan</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>12 - 14 Okt</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>Hasbi &amp; Dina</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>Kontak 11 Kosma angkatan 2026 terkumpul 100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Sosialisasi Maba</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Pemetaan Jadwal Kosong Kelas Maba</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>14 - 16 Okt</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Hasbi &amp; Dina</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>Jadwal jam kosong 11 prodi terkumpul &amp; dipetakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Sosialisasi Maba</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Penyebaran Poster Pendaftaran LDKM ke Grup KPAM</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>14 - 18 Okt</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Tim Humas</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Poster disebar, menjawab kendala sertifikat KPAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Sosialisasi Maba</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Eksekusi Sosialisasi Masuk Kelas Maba (Roadshow)</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>19 - 23 Okt</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>Hasbi, Dina, Klar, Rina</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Sedang Berjalan</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>BK &amp; PBI selesai (Done), 9 prodi lain berjalan sesuai jadwal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Sosialisasi Maba</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Edukasi &amp; Follow-up Pendaftaran Maba (Solusi KPAM)</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>19 - 24 Okt</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Tim Humas</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Sedang Berjalan</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>Maba diyakinkan tetap daftar walau sertif KPAM belum turun</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Pengumpulan Opsi Kandidat Narasumber (4 Topik)</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>12 - 16 Okt</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Tim Humas</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>3 Dosen Internal (Pak Ade, Pak Yudhy, Pak Miki) &amp; 2 Eksternal (Zen RS, Fathimah UI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Penyelarasan TOR dengan Divisi Acara</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>16 - 18 Okt</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Dina &amp; Div. Acara</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>TOR resmi LDKM 2026 terbit (Tema: Dari Gagasan Menjadi Gerakan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Pengiriman Surat Undangan &amp; TOR ke Calon Pemateri</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>19 - 20 Okt</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>LO / PIC Pemateri</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Sedang Berjalan</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>Mulai hubungi calon pemateri internal &amp; eksternal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Fiksasi 4 Pemateri LDKM (Konfirmasi Kesediaan)</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>19 - 21 Okt</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Dina &amp; PIC Pemateri</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Sedang Berjalan</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Batas maksimal fiksasi tanggal 21 Okt</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Pengumpulan Berkas Pemateri (CV, Foto Formal, PPT)</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>21 - 24 Okt</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>LO / PIC Pemateri</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Berkas untuk publikasi PDD dan bahan moderator</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Narasumber</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Konfirmasi Teknis Sesi (Jadwal, Durasi, Ruangan, Format)</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>24 - 26 Okt</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>LO Humas &amp; Acara</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Kepastian teknis H-3 acara</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Perizinan Ruangan</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Pengajuan Awal Peminjaman Ruangan ke Sarpras</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>12 - 16 Okt</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>Tilka (Koor Sekre)</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>Selesai</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Koordinasi awal aula dan ruang kelas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Perizinan Ruangan</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Fiksasi Ruang Peserta FKOM (201-208) &amp; P3K (213) ke Bu Atat</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>19 - 21 Okt</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Tilka</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Sedang Berjalan</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Menindaklanjuti hasil rapat 16 Okt ke Bu Atat</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Perizinan Ruangan</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Kepastian Izin Ruang Transit Pemateri &amp; Ruang Panitia</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>21 - 23 Okt</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Tilka</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Ruang transit pemateri dan panitia lantai bawah</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Hari-H LDKM</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Briefing Teknis LO Humas Pendamping Pemateri</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>27 - 28 Okt</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Tim Humas</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>Gladi kotor &amp; pemantapan tugas LO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Hari-H LDKM</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Pendampingan Pemateri Day 1 (Kamis, 29 Okt - Aula)</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>29 Okt</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>LO Humas</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 1 &amp; 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Hari-H LDKM</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Pendampingan Pemateri Day 2 (Jumat, 30 Okt - Aula)</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>30 Okt</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>LO Humas</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 3 &amp; 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Hari-H LDKM</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Pendampingan Tamu Alumni Day 3 (Sabtu, 31 Okt - Villa)</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>31 Okt</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>LO Humas</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Belum Mulai</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>Hospitality sesi sharing alumni &amp; penutupan acara</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: terapkan desain minimalis modern dan pewarnaan status di sheet 5. Timeline Humas
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <color rgb="FF262626"/>
@@ -77,8 +77,37 @@
       <color rgb="007F6000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -128,8 +157,44 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -243,11 +308,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -296,6 +375,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2543,705 +2646,714 @@
   </sheetPr>
   <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="20" t="inlineStr">
         <is>
           <t>Pilar Kerja</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="20" t="inlineStr">
         <is>
           <t>Program Kerja / Tugas Spesifik</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="20" t="inlineStr">
         <is>
           <t>Rentang Waktu</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="20" t="inlineStr">
         <is>
           <t>PIC / Petugas</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="20" t="inlineStr">
         <is>
           <t>Keterangan / Output yang Diharapkan</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Pendataan Kontak Kosma 11 Jurusan</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>12 - 14 Okt</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>Hasbi &amp; Dina</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Kontak 11 Kosma angkatan 2026 terkumpul 100%</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="25" t="inlineStr">
         <is>
           <t>Pemetaan Jadwal Kosong Kelas Maba</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>14 - 16 Okt</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>Hasbi &amp; Dina</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="G3" s="25" t="inlineStr">
         <is>
           <t>Jadwal jam kosong 11 prodi terkumpul &amp; dipetakan</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Penyebaran Poster Pendaftaran LDKM ke Grup KPAM</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>14 - 18 Okt</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Poster disebar, menjawab kendala sertifikat KPAM</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Eksekusi Sosialisasi Masuk Kelas Maba (Roadshow)</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>19 - 23 Okt</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>Hasbi, Dina, Klar, Rina</t>
         </is>
       </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="26" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
         <is>
           <t>BK &amp; PBI selesai (Done), 9 prodi lain berjalan sesuai jadwal</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Edukasi &amp; Follow-up Pendaftaran Maba (Solusi KPAM)</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>19 - 24 Okt</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Maba diyakinkan tetap daftar walau sertif KPAM belum turun</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Pengumpulan Opsi Kandidat Narasumber (4 Topik)</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>12 - 16 Okt</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
         <is>
           <t>3 Dosen Internal (Pak Ade, Pak Yudhy, Pak Miki) &amp; 2 Eksternal (Zen RS, Fathimah UI)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Penyelarasan TOR dengan Divisi Acara</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>16 - 18 Okt</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Dina &amp; Div. Acara</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>TOR resmi LDKM 2026 terbit (Tema: Dari Gagasan Menjadi Gerakan)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Pengiriman Surat Undangan &amp; TOR ke Calon Pemateri</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>19 - 20 Okt</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>LO / PIC Pemateri</t>
         </is>
       </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="G9" s="25" t="inlineStr">
         <is>
           <t>Mulai hubungi calon pemateri internal &amp; eksternal</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Fiksasi 4 Pemateri LDKM (Konfirmasi Kesediaan)</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>19 - 21 Okt</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Dina &amp; PIC Pemateri</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F10" s="26" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="22" t="inlineStr">
         <is>
           <t>Batas maksimal fiksasi tanggal 21 Okt</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Pengumpulan Berkas Pemateri (CV, Foto Formal, PPT)</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>21 - 24 Okt</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>LO / PIC Pemateri</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="G11" s="25" t="inlineStr">
         <is>
           <t>Berkas untuk publikasi PDD dan bahan moderator</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Konfirmasi Teknis Sesi (Jadwal, Durasi, Ruangan, Format)</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>24 - 26 Okt</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>LO Humas &amp; Acara</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>Kepastian teknis H-3 acara</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>Pengajuan Awal Peminjaman Ruangan ke Sarpras</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>12 - 16 Okt</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Tilka (Koor Sekre)</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G13" s="25" t="inlineStr">
         <is>
           <t>Koordinasi awal aula dan ruang kelas</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Fiksasi Ruang Peserta FKOM (201-208) &amp; P3K (213) ke Bu Atat</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>19 - 21 Okt</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>Tilka</t>
         </is>
       </c>
-      <c r="F14" s="19" t="inlineStr">
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>Menindaklanjuti hasil rapat 16 Okt ke Bu Atat</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Kepastian Izin Ruang Transit Pemateri &amp; Ruang Panitia</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>21 - 23 Okt</t>
         </is>
       </c>
-      <c r="E15" s="17" t="inlineStr">
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t>Tilka</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="G15" s="25" t="inlineStr">
         <is>
           <t>Ruang transit pemateri dan panitia lantai bawah</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Briefing Teknis LO Humas Pendamping Pemateri</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>27 - 28 Okt</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Gladi kotor &amp; pemantapan tugas LO</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t>Pendampingan Pemateri Day 1 (Kamis, 29 Okt - Aula)</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>29 Okt</t>
         </is>
       </c>
-      <c r="E17" s="17" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="G17" s="25" t="inlineStr">
         <is>
           <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 1 &amp; 2</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>Pendampingan Pemateri Day 2 (Jumat, 30 Okt - Aula)</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>30 Okt</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
         <is>
           <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 3 &amp; 4</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="25" t="inlineStr">
         <is>
           <t>Pendampingan Tamu Alumni Day 3 (Sabtu, 31 Okt - Villa)</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>31 Okt</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="G19" s="25" t="inlineStr">
         <is>
           <t>Hospitality sesi sharing alumni &amp; penutupan acara</t>
         </is>

</xml_diff>

<commit_message>
update: alokasi pemateri baru (Topik 1 khusus Zen RS Eksternal, Topik 2-3 Internal, Topik 4 Eksternal)
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Internal</t>
+          <t>Eksternal</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1116,18 +1116,22 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
+          <t>Zen RS (Zen Rachmat Sugito)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Dosen Internal Kampus</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="n"/>
+          <t>Penulis / Jurnalis Senior / Literasi</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>@zen.rs</t>
+        </is>
+      </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Ikut RAB Kampus</t>
+          <t>Cek Rate Card</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -1223,7 +1227,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Eksternal</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1233,20 +1237,24 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Zen RS (Zen Rachmat Sugito)</t>
+          <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Penulis / Jurnalis Senior / Literasi</t>
+          <t>Dosen Internal Kampus</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>@zen.rs</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Ikut RAB Kampus</t>
+        </is>
+      </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Belum</t>
@@ -1261,10 +1269,26 @@
           <t>Opsi 2</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Pak Yudhy (Dr. Yudhy, Drs., M.Ag.)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Dosen Internal Kampus</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Ikut RAB Kampus</t>
+        </is>
+      </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Belum</t>
@@ -1279,10 +1303,26 @@
           <t>Opsi 3</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Dosen Internal Kampus</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Ikut RAB Kampus</t>
+        </is>
+      </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Belum</t>
@@ -1334,7 +1374,11 @@
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F20" s="3" t="n"/>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
@@ -1364,7 +1408,11 @@
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
@@ -1394,7 +1442,11 @@
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>

</xml_diff>

<commit_message>
update: pemateri Topik 4 dari mitra IHLL (nama menyusul)
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -1495,20 +1495,24 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Fathimah Azzahra</t>
+          <t>Pemateri dari IHLL (Indonesia Humanitarian Logistics Lab)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Wakil Ketua BEM UI 2026</t>
+          <t>Mitra Lembaga IHLL</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>@fathimahzzhr</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="n"/>
+          <t>Menunggu Konfirmasi Nama</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Kerjasama Mitra / MoU</t>
+        </is>
+      </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Belum</t>

</xml_diff>

<commit_message>
feat: catat fiksasi Pak Yudhy (Topik 2 Mindset - Kamis 29 Okt) dan tindak lanjut permohonan beliau
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -1291,7 +1291,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Lolos / FIX</t>
         </is>
       </c>
     </row>
@@ -1725,18 +1725,26 @@
 (Fondasi)</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Eksternal</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Zen RS (Zen Rachmat Sugito)</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="10" t="n"/>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Proses Hubungi</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1784,28 +1792,44 @@
 (Mindset)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="10" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Yudhy, Drs., M.Ag. (Pak Yudhy)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Dosen Internal Kampus</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Tim Humas</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Bersedia (FIX) - Kamis 29 Okt (Pagi/Siang)</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Proses Sekre (Pak Yudi minta Proposal &amp; Surat)</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Req: Mau ngobrol dg Ketuplak</t>
         </is>
       </c>
     </row>
@@ -1843,18 +1867,26 @@
 (Kolaborasi)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Opsi: Pak Ade Iskandar / Pak Miki</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="10" t="n"/>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Menunggu Hubungi</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1902,18 +1934,26 @@
 (Ekspresi &amp; Aksi)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n"/>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Eksternal</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Pemateri dari Mitra IHLL</t>
+        </is>
+      </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="10" t="n"/>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Proses Acara</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">

</xml_diff>

<commit_message>
update: tambahkan opsi Pak Revi untuk Topik 3 (Kolaborasi Internal)
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Pak Yudhy (Dr. Yudhy, Drs., M.Ag.)</t>
+          <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
+          <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1434,12 +1434,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
+          <t>Pak Revi (Revi Nur Ridwan, M.Pd.)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Dosen Internal Kampus</t>
+          <t>Dosen Internal Kampus (PBI/FKIP)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Opsi: Pak Ade Iskandar / Pak Miki</t>
+          <t>Opsi: Pak Miki / Pak Ade / Pak Revi</t>
         </is>
       </c>
       <c r="E8" s="3" t="n"/>

</xml_diff>

<commit_message>
update: jadwal sosialisasi Selasa 20 Okt untuk Teknik Industri (B203) dan Teknologi Pangan (B413)
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -2295,17 +2295,17 @@
       </c>
       <c r="F2" s="17" t="inlineStr">
         <is>
-          <t>Rabu (09.10-10.00) &amp; Kamis (10.50-13.00)</t>
+          <t>Selasa (10.10 di B203)</t>
         </is>
       </c>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t>Ada Jadwal</t>
+          <t>Terjadwal Besok</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dina</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>Rabu (12.20) &amp; Jumat (09.20-09.50)</t>
+          <t>Selasa (11.30 di B413)</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Ada Jadwal</t>
+          <t>Terjadwal Besok</t>
         </is>
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Dina</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: 4 prodi selesai sosialisasi (TI, BD, Ag, TP) total 6 dari 11 selesai
</commit_message>
<xml_diff>
--- a/Rekap & Tracker Humas LDKM 2026.xlsx
+++ b/Rekap & Tracker Humas LDKM 2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="600" firstSheet="1" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Opsi Kandidat" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <color rgb="FF262626"/>
@@ -58,7 +58,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -68,46 +68,34 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00375623"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="007F6000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="001E293B"/>
+      <color rgb="FF1E293B"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00166534"/>
+      <color rgb="FF166534"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="FF92400E"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0064748B"/>
+      <color rgb="FF64748B"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -141,56 +129,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FF1E293B"/>
+        <bgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -215,15 +191,6 @@
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -256,26 +223,6 @@
       <top style="thin">
         <color rgb="FFD9D9D9"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
@@ -296,49 +243,74 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </left>
       <right style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </right>
       <top style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -349,57 +321,66 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -812,17 +793,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>A. ACUAN 4 TOPIK MATERI (2 TOPIK INTERNAL &amp; 2 TOPIK EKSTERNAL)</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="12" t="n"/>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="20" t="n"/>
+      <c r="E1" s="20" t="n"/>
+      <c r="F1" s="20" t="n"/>
+      <c r="G1" s="21" t="n"/>
     </row>
     <row r="2" ht="26.1" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -862,156 +843,156 @@
       </c>
     </row>
     <row r="3" ht="21.95" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Acuan topik untuk calon pemateri</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Pilih: Internal / Eksternal</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Cth: Kamis, 29 Okt (09.00-10.30)</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Cth: Rp 300.000 / Plakat</t>
         </is>
       </c>
     </row>
     <row r="4" ht="33.95" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Fondasi</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Kepemimpinan &amp; Manajemen Organisasi (KMO)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Prinsip kepemimpinan, fungsi organisasi, pembagian peran, tanggung jawab, dan kerja tim.</t>
         </is>
       </c>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22" t="n"/>
     </row>
     <row r="5" ht="33.95" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Mindset</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Self-Awareness &amp; Critical Thinking</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Potensi &amp; nilai diri, berpikir kritis, analisis masalah, serta memahami tujuan setiap instruksi.</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="22" t="n"/>
     </row>
     <row r="6" ht="33.95" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Kolaborasi</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>Collaboration, Solidarity &amp; Conflict Management</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Empati, kepercayaan, mengelola konflik, dan penyelesaian masalah bersama.</t>
         </is>
       </c>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22" t="n"/>
     </row>
     <row r="7" ht="33.95" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Ekspresi &amp; Aksi</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Effective Communication, Assertiveness &amp; Public Speaking</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Menyampaikan ide dengan jelas, menyusun argumen, berani berpendapat, dan menyuarakan aspirasi.</t>
         </is>
       </c>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="22" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1"/>
     <row r="9" ht="27.95" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>B. DAFTAR OPSI KANDIDAT (TIAP TOPIK 4 OPSI PEMATERI)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="12" t="n"/>
+      <c r="B9" s="20" t="n"/>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="20" t="n"/>
+      <c r="E9" s="20" t="n"/>
+      <c r="F9" s="20" t="n"/>
+      <c r="G9" s="20" t="n"/>
+      <c r="H9" s="21" t="n"/>
     </row>
     <row r="10" ht="26.1" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
@@ -1056,518 +1037,518 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Isi: Internal / Eksternal</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>1 s.d. 4</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Tulis nama lengkap &amp; gelar</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Cth: Dosen Prodi X / Presma BEM Y</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Cth: 0812xxx / @username</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Cth: Ikut RAB / Rp 300rb</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Isi: Belum / Lolos / Cadangan / Coret</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26.1" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>1. KMO
 (Fondasi)</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Eksternal</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Opsi 1</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Zen RS (Zen Rachmat Sugito)</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Penulis / Jurnalis Senior / Literasi</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>@zen.rs</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>Cek Rate Card</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26.1" customHeight="1">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="23" t="n"/>
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Opsi 2</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Pak Yudhy (Dr. Yudhy, Drs., M.Ag.)</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26.1" customHeight="1">
-      <c r="A14" s="13" t="n"/>
-      <c r="B14" s="13" t="n"/>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="23" t="n"/>
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Opsi 3</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26.1" customHeight="1">
-      <c r="A15" s="14" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="A15" s="24" t="n"/>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Opsi 4</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="22" t="n"/>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26.1" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>2. Self-Awareness &amp; Critical Thinking
 (Mindset)</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Opsi 1</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26.1" customHeight="1">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Opsi 2</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Pak Yudhy (Dr. Yudhy, Drs., M.Ag.)</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Lolos / FIX</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26.1" customHeight="1">
-      <c r="A18" s="13" t="n"/>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>Opsi 3</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26.1" customHeight="1">
-      <c r="A19" s="14" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="A19" s="24" t="n"/>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>Opsi 4</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="22" t="n"/>
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26.1" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>3. Collaboration &amp; Conflict Mgmt
 (Kolaborasi)</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>Opsi 1</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Pak Miki (Miki Wijaya, M.Kom.)</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26.1" customHeight="1">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>Opsi 2</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Pak Ade Iskandar (Ade Iskandar Nasution, S.H., M.H.)</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26.1" customHeight="1">
-      <c r="A22" s="13" t="n"/>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="22" t="inlineStr">
         <is>
           <t>Opsi 3</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Pak Revi (Revi Nur Ridwan, M.Pd.)</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus (PBI/FKIP)</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="G22" s="22" t="inlineStr">
         <is>
           <t>Ikut RAB Kampus</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26.1" customHeight="1">
-      <c r="A23" s="14" t="n"/>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>Opsi 4</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26.1" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>4. Communication &amp; Public Speaking
 (Ekspresi &amp; Aksi)</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>Eksternal</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>Opsi 1</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Pemateri dari IHLL (Indonesia Humanitarian Logistics Lab)</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Mitra Lembaga IHLL</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Menunggu Konfirmasi Nama</t>
         </is>
       </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="G24" s="22" t="inlineStr">
         <is>
           <t>Kerjasama Mitra / MoU</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26.1" customHeight="1">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>Opsi 2</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="22" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26.1" customHeight="1">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="23" t="n"/>
+      <c r="C26" s="22" t="inlineStr">
         <is>
           <t>Opsi 3</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="22" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26.1" customHeight="1">
-      <c r="A27" s="14" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="A27" s="24" t="n"/>
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>Opsi 4</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="10" t="n"/>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="22" t="n"/>
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
@@ -1610,19 +1591,19 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>TRACKER PEMATERI TERPILIH (2 TOPIK INTERNAL &amp; 2 TOPIK EKSTERNAL)</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="11" t="n"/>
-      <c r="H1" s="11" t="n"/>
-      <c r="I1" s="12" t="n"/>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="20" t="n"/>
+      <c r="E1" s="20" t="n"/>
+      <c r="F1" s="20" t="n"/>
+      <c r="G1" s="20" t="n"/>
+      <c r="H1" s="20" t="n"/>
+      <c r="I1" s="21" t="n"/>
     </row>
     <row r="2" ht="26.1" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -1672,323 +1653,323 @@
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Isi: Internal / Eksternal</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Utama / Cadangan</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Nama kandidat lolos filter</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>No. WA / CP</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Nama LO Humas</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Isi: Belum / Sudah Chat / Bersedia / Batal</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Isi: Belum / Proses Sekre / Terkirim</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Isi: Belum / Sebagian / Lengkap</t>
         </is>
       </c>
     </row>
     <row r="4" ht="27.95" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>1. KMO
 (Fondasi)</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Eksternal</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Zen RS (Zen Rachmat Sugito)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Proses Hubungi</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="5" ht="27.95" customHeight="1">
-      <c r="A5" s="14" t="n"/>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Cadangan</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Standby</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="6" ht="27.95" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>2. Self-Awareness &amp; Critical Thinking
 (Mindset)</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Dr. Yudhy, Drs., M.Ag. (Pak Yudhy)</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Dosen Internal Kampus</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Bersedia (FIX) - Kamis 29 Okt (Pagi/Siang)</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Proses Sekre (Pak Yudi minta Proposal &amp; Surat)</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Req: Mau ngobrol dg Ketuplak</t>
         </is>
       </c>
     </row>
     <row r="7" ht="27.95" customHeight="1">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="A7" s="24" t="n"/>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Cadangan</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Standby</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="8" ht="27.95" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>3. Collaboration &amp; Conflict Mgmt
 (Kolaborasi)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Internal</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Opsi: Pak Miki / Pak Ade / Pak Revi</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Menunggu Hubungi</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="9" ht="27.95" customHeight="1">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="A9" s="24" t="n"/>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Cadangan</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Standby</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="10" ht="27.95" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>4. Communication &amp; Public Speaking
 (Ekspresi &amp; Aksi)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Eksternal</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Utama</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Pemateri dari Mitra IHLL</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Proses Acara</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Belum</t>
         </is>
       </c>
     </row>
     <row r="11" ht="27.95" customHeight="1">
-      <c r="A11" s="14" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="A11" s="24" t="n"/>
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Cadangan</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Standby</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2025,13 +2006,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>TIPS SINGKAT &amp; TEMPLATE CHAT HUMAS</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="12" t="n"/>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="21" t="n"/>
     </row>
     <row r="2" ht="26.1" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -2051,17 +2032,17 @@
       </c>
     </row>
     <row r="3" ht="75" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Tips Chat Humas</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>Aturan Dasar</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>1. Chat di jam sopan (08.00 - 17.00 WIB).
 2. Gunakan foto profil WA yang jelas &amp; nama asli.
@@ -2071,18 +2052,18 @@
       </c>
     </row>
     <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>1. Cek Rate Card
 (Sebelum Filter)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Pemateri Eksternal / CP / Manajer</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Selamat [pagi/siang/sore] Kak/Bapak/Ibu [Nama],
 Perkenalkan saya [Nama Kamu] dari Humas LDKM BEM [Nama Kampus] 2026.
@@ -2093,18 +2074,18 @@
       </c>
     </row>
     <row r="5" ht="195" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>2. Undangan Pemateri
 Internal</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Dosen / Pihak Kampus</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Assalamualaikum wr. wb. / Selamat [pagi/siang/sore] Bapak/Ibu [Nama Dosen],
 Mohon maaf mengganggu waktunya. Saya [Nama Kamu] dari Humas LDKM BEM [Nama Kampus] 2026 bermaksud memohon kesediaan Bapak/Ibu untuk menjadi Pemateri LDKM pada:
@@ -2118,18 +2099,18 @@
       </c>
     </row>
     <row r="6" ht="210" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>3. Undangan Pemateri
 Eksternal</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Alumni / BEM Luar / Praktisi</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Selamat [pagi/siang/sore] Kak [Nama],
 Perkenalkan saya [Nama Kamu] dari Humas LDKM BEM [Nama Kampus] 2026.
@@ -2144,18 +2125,18 @@
       </c>
     </row>
     <row r="7" ht="180" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>4. Kirim Surat, TOR
 &amp; Minta CV/PPT</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Pemateri yang Sudah Bersedia</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Selamat [pagi/siang/sore] Bapak/Ibu/Kak [Nama],
 Terima kasih atas kesediaannya menjadi pemateri LDKM BEM 2026. Berikut kami lampirkan Surat Undangan Resmi dan TOR Materi.
@@ -2168,18 +2149,18 @@
       </c>
     </row>
     <row r="8" ht="135" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>5. Follow-Up
 Kesediaan</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Kandidat Belum Membalas</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Selamat [pagi/siang/sore] Bapak/Ibu/Kak [Nama],
 Mohon maaf mengganggu waktunya kembali. Saya [Nama Kamu] dari Humas LDKM BEM 2026 izin menindaklanjuti pesan sebelumnya terkait permohonan sebagai narasumber pada [Tanggal].
@@ -2189,18 +2170,18 @@
       </c>
     </row>
     <row r="9" ht="120" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>6. Peminjaman
 Ruangan</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Bagian Sarpras / Ruangan Kampus</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Selamat [pagi/siang/sore] Bapak/Ibu [Nama],
 Perkenalkan saya [Nama] dari Humas LDKM BEM 2026. Sehubungan dengan kegiatan LDKM pada 29–31 Oktober 2026, kami izin menanyakan ketersediaan ruangan [Nama Ruangan] pada tanggal tersebut. Untuk surat peminjaman resmi sedang dalam proses pengajuan.
@@ -2225,505 +2206,505 @@
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="16.5" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Jurusan</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Nama Kosma</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>Kontak WA</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>PIC Humas</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>Waktu Luang / Jadwal Kelas</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="8" t="inlineStr">
         <is>
           <t>Status Chat</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="8" t="inlineStr">
         <is>
           <t>Petugas Sosialisasi (Kondisional)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Teknik Industri</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Royyan</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>+62 838-7551-6303</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Hasbi</t>
         </is>
       </c>
-      <c r="F2" s="17" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>Selasa (10.10 di B203)</t>
         </is>
       </c>
-      <c r="G2" s="16" t="inlineStr">
-        <is>
-          <t>Terjadwal Besok</t>
-        </is>
-      </c>
-      <c r="H2" s="17" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>Dina</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Teknik Informatika</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Siraj</t>
         </is>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>+62 822-9883-1441</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Hasbi</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>Senin (11.30-an) &amp; Rabu (09.10-an)</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Ada Jadwal</t>
         </is>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Agribisnis</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Marsya</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>+62 812-2407-3226</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Hasbi</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Jumat (10.30) &amp; Hari ini (s/d 14.00 kosong)</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Dina, Klar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Teknologi Pangan</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Isra</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>+62 895-3298-97079</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Hasbi</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Selasa (11.30 di B413)</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Bimbingan Konseling</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>+62 813-3087-7193</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Hasbi</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Rina</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Pendidikan Bahasa Inggris</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>+62 823-3841-3830</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Jumat (10.50-an)</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Dina, Klar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Perbankan Syariah</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Yasir</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>+62 838-2427-2554</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Belum Ada Jadwal</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Manajemen Bisnis Syariah</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Jumat (10.00-an)</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Ada Jadwal</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Teknologi Pangan</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>Isra</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>+62 895-3298-97079</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>Hasbi</t>
-        </is>
-      </c>
-      <c r="F5" s="17" t="inlineStr">
-        <is>
-          <t>Selasa (11.30 di B413)</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr">
-        <is>
-          <t>Terjadwal Besok</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Bisnis Digital</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Saepul</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>+62 851-3371-6189</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Dina</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Bimbingan Konseling</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Selasa (10.10-13.20)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Selesai (Done)</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Komputerisasi Akuntansi</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Nurul</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>+62 822-6285-6159</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Dina</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Jumat (10.00), Selasa (13.30), Kamis (08.00-13.20 &amp; 15.00)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Ada Jadwal</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>+62 813-3087-7193</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Hasbi</t>
-        </is>
-      </c>
-      <c r="F6" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>Selesai (Done)</t>
-        </is>
-      </c>
-      <c r="H6" s="17" t="inlineStr">
-        <is>
-          <t>Rina</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Pendidikan Bahasa Inggris</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="inlineStr">
-        <is>
-          <t>+62 823-3841-3830</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Sistem Informasi</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Raka</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>+62 831-4563-3721</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Dina</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>Jumat (10.50-an)</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
-        <is>
-          <t>Selesai (Done)</t>
-        </is>
-      </c>
-      <c r="H7" s="17" t="inlineStr">
-        <is>
-          <t>Dina, Klar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Perbankan Syariah</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>Yasir</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>+62 838-2427-2554</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>Dina</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>Belum Ada Jadwal</t>
-        </is>
-      </c>
-      <c r="H8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Manajemen Bisnis Syariah</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Dina</t>
-        </is>
-      </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>Jumat (10.00-an)</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Senin (10.10-13.30)</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Ada Jadwal</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Bisnis Digital</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>Saepul</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>+62 851-3371-6189</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>Dina</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>Selasa (10.10-13.20)</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>Ada Jadwal</t>
-        </is>
-      </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Komputerisasi Akuntansi</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="inlineStr">
-        <is>
-          <t>Nurul</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>+62 822-6285-6159</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>Dina</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>Jumat (10.00), Selasa (13.30), Kamis (08.00-13.20 &amp; 15.00)</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>Ada Jadwal</t>
-        </is>
-      </c>
-      <c r="H11" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Sistem Informasi</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>Raka</t>
-        </is>
-      </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>+62 831-4563-3721</t>
-        </is>
-      </c>
-      <c r="E12" s="16" t="inlineStr">
-        <is>
-          <t>Dina</t>
-        </is>
-      </c>
-      <c r="F12" s="17" t="inlineStr">
-        <is>
-          <t>Senin (10.10-13.30)</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>Ada Jadwal</t>
-        </is>
-      </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2745,711 +2726,711 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="53.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="15.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+    <row r="1" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Pilar Kerja</t>
         </is>
       </c>
-      <c r="C1" s="20" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Program Kerja / Tugas Spesifik</t>
         </is>
       </c>
-      <c r="D1" s="20" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Rentang Waktu</t>
         </is>
       </c>
-      <c r="E1" s="20" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>PIC / Petugas</t>
         </is>
       </c>
-      <c r="F1" s="20" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="20" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Keterangan / Output yang Diharapkan</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+    <row r="2" ht="21.95" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Pendataan Kontak Kosma 11 Jurusan</t>
         </is>
       </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>12 - 14 Okt</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Hasbi &amp; Dina</t>
         </is>
       </c>
-      <c r="F2" s="23" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Kontak 11 Kosma angkatan 2026 terkumpul 100%</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
+    <row r="3" ht="21.95" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C3" s="25" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>Pemetaan Jadwal Kosong Kelas Maba</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>14 - 16 Okt</t>
         </is>
       </c>
-      <c r="E3" s="25" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Hasbi &amp; Dina</t>
         </is>
       </c>
-      <c r="F3" s="23" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G3" s="25" t="inlineStr">
+      <c r="G3" s="16" t="inlineStr">
         <is>
           <t>Jadwal jam kosong 11 prodi terkumpul &amp; dipetakan</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+    <row r="4" ht="21.95" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Penyebaran Poster Pendaftaran LDKM ke Grup KPAM</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>14 - 18 Okt</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G4" s="22" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Poster disebar, menjawab kendala sertifikat KPAM</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+    <row r="5" ht="21.95" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Eksekusi Sosialisasi Masuk Kelas Maba (Roadshow)</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>19 - 23 Okt</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Hasbi, Dina, Klar, Rina</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>BK &amp; PBI selesai (Done), 9 prodi lain berjalan sesuai jadwal</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+    <row r="6" ht="21.95" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Sosialisasi Maba</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Edukasi &amp; Follow-up Pendaftaran Maba (Solusi KPAM)</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>19 - 24 Okt</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G6" s="22" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Maba diyakinkan tetap daftar walau sertif KPAM belum turun</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="7" ht="21.95" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Pengumpulan Opsi Kandidat Narasumber (4 Topik)</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>12 - 16 Okt</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>3 Dosen Internal (Pak Ade, Pak Yudhy, Pak Miki) &amp; 2 Eksternal (Zen RS, Fathimah UI)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+    <row r="8" ht="21.95" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Penyelarasan TOR dengan Divisi Acara</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>16 - 18 Okt</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Dina &amp; Div. Acara</t>
         </is>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G8" s="22" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>TOR resmi LDKM 2026 terbit (Tema: Dari Gagasan Menjadi Gerakan)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
+    <row r="9" ht="21.95" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Pengiriman Surat Undangan &amp; TOR ke Calon Pemateri</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>19 - 20 Okt</t>
         </is>
       </c>
-      <c r="E9" s="25" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>LO / PIC Pemateri</t>
         </is>
       </c>
-      <c r="F9" s="26" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G9" s="25" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Mulai hubungi calon pemateri internal &amp; eksternal</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+    <row r="10" ht="21.95" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Fiksasi 4 Pemateri LDKM (Konfirmasi Kesediaan)</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>19 - 21 Okt</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Dina &amp; PIC Pemateri</t>
         </is>
       </c>
-      <c r="F10" s="26" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G10" s="22" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Batas maksimal fiksasi tanggal 21 Okt</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+    <row r="11" ht="21.95" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Pengumpulan Berkas Pemateri (CV, Foto Formal, PPT)</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>21 - 24 Okt</t>
         </is>
       </c>
-      <c r="E11" s="25" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>LO / PIC Pemateri</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G11" s="25" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Berkas untuk publikasi PDD dan bahan moderator</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+    <row r="12" ht="21.95" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Narasumber</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Konfirmasi Teknis Sesi (Jadwal, Durasi, Ruangan, Format)</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>24 - 26 Okt</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>LO Humas &amp; Acara</t>
         </is>
       </c>
-      <c r="F12" s="27" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Kepastian teknis H-3 acara</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
+    <row r="13" ht="21.95" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Pengajuan Awal Peminjaman Ruangan ke Sarpras</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>12 - 16 Okt</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Tilka (Koor Sekre)</t>
         </is>
       </c>
-      <c r="F13" s="23" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Selesai</t>
         </is>
       </c>
-      <c r="G13" s="25" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Koordinasi awal aula dan ruang kelas</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+    <row r="14" ht="21.95" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Fiksasi Ruang Peserta FKOM (201-208) &amp; P3K (213) ke Bu Atat</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>19 - 21 Okt</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>Tilka</t>
         </is>
       </c>
-      <c r="F14" s="26" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>Sedang Berjalan</t>
         </is>
       </c>
-      <c r="G14" s="22" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Menindaklanjuti hasil rapat 16 Okt ke Bu Atat</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+    <row r="15" ht="21.95" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Perizinan Ruangan</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Kepastian Izin Ruang Transit Pemateri &amp; Ruang Panitia</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>21 - 23 Okt</t>
         </is>
       </c>
-      <c r="E15" s="25" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>Tilka</t>
         </is>
       </c>
-      <c r="F15" s="27" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G15" s="25" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Ruang transit pemateri dan panitia lantai bawah</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="16" ht="21.95" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Briefing Teknis LO Humas Pendamping Pemateri</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>27 - 28 Okt</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>Tim Humas</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G16" s="22" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Gladi kotor &amp; pemantapan tugas LO</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+    <row r="17" ht="21.95" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C17" s="25" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>Pendampingan Pemateri Day 1 (Kamis, 29 Okt - Aula)</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>29 Okt</t>
         </is>
       </c>
-      <c r="E17" s="25" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F17" s="27" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G17" s="25" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 1 &amp; 2</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+    <row r="18" ht="21.95" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C18" s="22" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>Pendampingan Pemateri Day 2 (Jumat, 30 Okt - Aula)</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>30 Okt</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F18" s="27" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G18" s="22" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>Penyambutan, ruang transit, konsumsi, plakat Pematerian 3 &amp; 4</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+    <row r="19" ht="21.95" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B19" s="24" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Hari-H LDKM</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>Pendampingan Tamu Alumni Day 3 (Sabtu, 31 Okt - Villa)</t>
         </is>
       </c>
-      <c r="D19" s="24" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>31 Okt</t>
         </is>
       </c>
-      <c r="E19" s="25" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>LO Humas</t>
         </is>
       </c>
-      <c r="F19" s="27" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>Belum Mulai</t>
         </is>
       </c>
-      <c r="G19" s="25" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>Hospitality sesi sharing alumni &amp; penutupan acara</t>
         </is>

</xml_diff>